<commit_message>
Create 4 SharePoint list templates as Excel tables
テーブル形式のExcelファイルを4つ生成：
- EQ_Config_Members.xlsx: スタッフ・マネージャー・管理者の名簿
- EQ_Received_Items.xlsx: エラーログ記録用
- EQ_Events.xlsx: イベント（地震）データ格納
- EQ_Responses.xlsx: 安否確認回答データ格納

Each file is formatted as a proper Excel Table so it can be imported
to SharePoint using the "Import from Excel" feature.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Er36jAyBsenGX9kWsBw39k
</commit_message>
<xml_diff>
--- a/power_automate_safety_checkin/EQ_Responses.xlsx
+++ b/power_automate_safety_checkin/EQ_Responses.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Responses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,24 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -136,6 +122,24 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EQ_ResponsesTable" displayName="EQ_ResponsesTable" ref="A1:I1" headerRowCount="1">
+  <autoFilter ref="A1:I1"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="EventID"/>
+    <tableColumn id="2" name="EmployeeID"/>
+    <tableColumn id="3" name="Email"/>
+    <tableColumn id="4" name="ResponseCode"/>
+    <tableColumn id="5" name="SafetyStatus"/>
+    <tableColumn id="6" name="WorkStatus"/>
+    <tableColumn id="7" name="RespondedAt"/>
+    <tableColumn id="8" name="Comment"/>
+    <tableColumn id="9" name="Revision"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -442,47 +446,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>EventID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>EmployeeID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ResponseCode</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SafetyStatus</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>WorkStatus</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>RespondedAt</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
@@ -490,5 +494,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild EQ_Responses.xlsx properly; fix missing Title column in flow spec
前回のEQ_Responses.xlsxはヘッダーのみで、SP_Get_Existing_Responseが
フィルターに使うTitle列が抜けていた(FLOW_LOGIC_SPEC.mdの記載にも不整合)。
Title=ResponseKeyを書き込み列に追加し、各列にコメントで想定型と説明を付与、
実例行とREADMEシートを追加した。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Er36jAyBsenGX9kWsBw39k
</commit_message>
<xml_diff>
--- a/power_automate_safety_checkin/EQ_Responses.xlsx
+++ b/power_automate_safety_checkin/EQ_Responses.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +28,43 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +72,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -124,19 +176,90 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>FLOW_LOGIC_SPEC.md</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+ResponseKeyを格納(EventID+'|'+EmployeeID)。SP_Get_Existing_Responseのフィルター対象。手入力しない(フローが自動生成)</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+対象イベントのID(EQ_EventsのTitleと同じ値)</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+回答者の社員ID(EQ_Config_MembersのTitleと同じ値)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+回答者のメールアドレス(T30対策の照合に使用)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+カードの選択値。'1'=無事出社可, '2'=無事出社不可, '3'=被災出社可, '4'=被災出社不可</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+ResponseCodeから変換。'Safe' または 'Affected'</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(1行)
+ResponseCodeから変換。'Available' または 'Unavailable'</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: 日付と時刻
+回答日時(UTC)。フローがutcNow()で自動設定</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: テキスト(複数行)
+回答者の任意コメント(最大500文字)</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>想定型: 数値
+同一回答者の再回答のたびに+1。初回作成時は1</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EQ_ResponsesTable" displayName="EQ_ResponsesTable" ref="A1:I1" headerRowCount="1">
-  <autoFilter ref="A1:I1"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="EventID"/>
-    <tableColumn id="2" name="EmployeeID"/>
-    <tableColumn id="3" name="Email"/>
-    <tableColumn id="4" name="ResponseCode"/>
-    <tableColumn id="5" name="SafetyStatus"/>
-    <tableColumn id="6" name="WorkStatus"/>
-    <tableColumn id="7" name="RespondedAt"/>
-    <tableColumn id="8" name="Comment"/>
-    <tableColumn id="9" name="Revision"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EQResponsesTable" displayName="EQResponsesTable" ref="A1:J2" headerRowCount="1">
+  <autoFilter ref="A1:J2"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Title"/>
+    <tableColumn id="2" name="EventID"/>
+    <tableColumn id="3" name="EmployeeID"/>
+    <tableColumn id="4" name="Email"/>
+    <tableColumn id="5" name="ResponseCode"/>
+    <tableColumn id="6" name="SafetyStatus"/>
+    <tableColumn id="7" name="WorkStatus"/>
+    <tableColumn id="8" name="RespondedAt"/>
+    <tableColumn id="9" name="Comment"/>
+    <tableColumn id="10" name="Revision"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -431,71 +554,197 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>EventID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>EmployeeID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ResponseCode</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>SafetyStatus</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>WorkStatus</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>RespondedAt</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EQ-20260731-090000-TOKYO|emp01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>EQ-20260731-090000-TOKYO</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>emp01</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>staff01@example.com</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Safe</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31 09:05:00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>自宅、特に被害なし</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>EQ_Responses.xlsx の使い方</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>1. 「Data」シートをSharePointの「Excelから新しいリストを作る」機能でアップロードしてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>2. 2行目(斜体グレーの実例行)は、列の中身をイメージしてもらうためのサンプルです。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SharePointへのアップロード後、リスト側でこの1件を削除してから運用を開始してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>3. 各列見出しにコメント(想定される型と説明)を付けています。セルにマウスを乗せると読めます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>4. Title列は、EventIDとEmployeeIDを '|' でつないだ値です。フロー(EQ04b_On_Response_DEV)が</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   重複回答チェックに使うため、削除・改名しないでください。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>